<commit_message>
Propagate IT corrections to EN dataset + fix IT footer garbage
Phase 1 (mechanical):
- Swapped answer_a/answer_b in 139 EN questions (2020) to match IT fix
- Stripped trailing colons from 215 EN fields (2017-2019)
- Fixed 33 IT answer_e fields with PDF page footer garbage
- Fixed 8 EN answer_e fields with partial footer artifacts

Phase 2 (API re-translation via claude-opus-4-8):
- Re-translated 73 fields across 59 questions where Italian text
  had semantic changes (2017, 2020-2023)
- Includes 5 previously missing answers for ssm2023574

Phase 3 (metadata):
- Updated translation_corrections.json (687 entries)
- Updated ITAMed_complete_EN_tracked.xlsx with highlighted changes

Total: 351 EN field modifications applied to all per-year + complete
JSON and XLSX files.
</commit_message>
<xml_diff>
--- a/Dataset/EN/xlsx/ITAMed_2017_EN.xlsx
+++ b/Dataset/EN/xlsx/ITAMed_2017_EN.xlsx
@@ -791,7 +791,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>The image shows an electrocardiographic tracing corresponding to:</t>
+          <t>The image shows an electrocardiographic tracing corresponding to</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>In relation to the image of the electrocardiographic tracing, the patient will most likely present with:</t>
+          <t>The patient will most likely present with</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>A 75-year-old patient is scheduled to undergo elective intestinal resection surgery. His medical history includes chronic atrial fibrillation treated with warfarin. According to current European guidelines, in preparation for surgery:</t>
+          <t>A 75-year-old patient is scheduled to undergo elective intestinal resection surgery. His medical history includes chronic atrial fibrillation treated with warfarin. According to current European guidelines, in preparation for surgery</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>A 54-year-old man is admitted to the intensive care unit with a diagnosis of septic shock of urinary tract origin. Hemodynamic support with vasoactive amines serves to:</t>
+          <t>A 54-year-old man is admitted to the intensive care unit with a diagnosis of septic shock of urinary tract origin. Hemodynamic support with vasoactive amines serves to</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>A 54-year-old patient has complained for 3 months of severe anal pain, triggered by defecation but persisting for several hours. At times he experiences mild rectal bleeding. To rule out the presence of other conditions that may cause rectal bleeding, also considering the patient's age, it is furthermore appropriate to perform as a first-line examination:</t>
+          <t>A 54-year-old patient has complained for 3 months of severe anal pain, triggered by defecation but persisting for several hours. At times he experiences mild rectal bleeding. To rule out the presence of other conditions that may cause rectal bleeding, also considering the patient's age, it is furthermore appropriate to perform as a first-line examination</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>A young couple presents to the gynecologist because they are unable to conceive. The first-line diagnostic workup should include:</t>
+          <t>A young couple presents to the gynecologist because they are unable to conceive. The first-line diagnostic workup should include</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -3325,7 +3325,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>A 32-year-old primiparous woman, with an unremarkable pre-pregnancy medical history, is diagnosed with moderate gestational hypertension. The patient contacts her gynecologist reporting that both her legs are swollen, but with no swelling in other locations. Based on what she has described over the phone, she is advised to:</t>
+          <t>A 32-year-old primiparous woman, with an unremarkable pre-pregnancy medical history, is diagnosed with moderate gestational hypertension. The patient contacts her gynecologist reporting that both her legs are swollen, but with no swelling in other locations. Based on what she has described over the phone, she is advised to</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>A 32-year-old primiparous woman, with an unremarkable pre-pregnancy medical history, is diagnosed with moderate gestational hypertension. The patient telephones her gynecologist complaining of abdominal pain after having eaten spoiled food. She is therefore advised to go to the nearest emergency department since, in view of her underlying condition, this symptom could bring the following conditions into the differential diagnosis:</t>
+          <t>A 32-year-old primiparous woman, with an unremarkable pre-pregnancy medical history, is diagnosed with moderate gestational hypertension. The patient telephones her gynecologist complaining of abdominal pain after having eaten spoiled food. She is therefore advised to go to the nearest emergency department since, in view of her underlying condition, this symptom could bring the following conditions into the differential diagnosis</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>A 42-year-old patient, gravida 3 para 0, is very frightened because a screening ultrasound at 32 weeks revealed an excess of amniotic fluid. The patient is informed that this condition is not very common and that:</t>
+          <t>A 42-year-old patient, gravida 3 para 0, is very frightened because a screening ultrasound at 32 weeks revealed an excess of amniotic fluid. The patient is informed that this condition is not very common and that</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -3557,7 +3557,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>In a case-control study to understand the etiology of esophageal cancer, 870 cases and 902 controls were investigated regarding the habitual consumption of spirits. The association between the disease and the risk factor can be quantified by calculating:</t>
+          <t>In a case-control study to understand the etiology of esophageal cancer, 870 cases and 902 controls were investigated regarding the habitual consumption of spirits. The association between the disease and the risk factor can be quantified by calculating</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -3625,7 +3625,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>In a case-control study to understand the etiology of esophageal cancer, 870 cases and 902 controls were investigated regarding the habitual consumption of spirits. Among the advantages of case-control studies, the following is generally indicated:</t>
+          <t>In a case-control study to understand the etiology of esophageal cancer, 870 cases and 902 controls were investigated regarding the habitual consumption of spirits. Among the advantages of case-control studies, the following is generally indicated</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -4157,7 +4157,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>A 48-year-old man, a smoker with hypertension treated with an ACE inhibitor, complains of epigastric pain for about 6 hours. The following parameters are recorded: BP 90/50 mmHg, HR 57/min, SpO2 99%, and an ECG is performed as shown in the figure. The abnormalities present are compatible with:</t>
+          <t>A 48-year-old man, a smoker with hypertension treated with an ACE inhibitor, complains of epigastric pain for about 6 hours. The following parameters are recorded: BP 90/50 mmHg, HR 57/min, SpO2 99%, and an ECG is performed as shown in the figure. The abnormalities present are compatible with</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -4225,7 +4225,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>A 48-year-old man, a smoker with hypertension on ACE inhibitor therapy, complains of epigastric pain for about 6 hours. The following parameters are recorded: BP 90/50 mmHg, HR 57/min, SpO2 99%, and an ECG is performed as shown in the figure. While the cath lab is being alerted, it is appropriate to begin administration of:</t>
+          <t>A 48-year-old man, a smoker with hypertension on ACE inhibitor therapy, complains of epigastric pain for about 6 hours. The following parameters are recorded: BP 90/50 mmHg, HR 57/min, SpO2 99%, and an ECG is performed as shown in the figure. While the cath lab is being alerted, it is appropriate to begin administration of</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -4293,7 +4293,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>A 48-year-old man, a smoker, hypertensive and on therapy with an ACE inhibitor. He complains of epigastric pain for about 6 hours. The following parameters are recorded: BP 90/50 mmHg, HR 57/min, SpO2 99%, and an ECG is performed as shown in the figure. The patient most likely has a lesion involving the:</t>
+          <t>A 48-year-old man, a smoker, hypertensive and on therapy with an ACE inhibitor. He complains of epigastric pain for about 6 hours. The following parameters are recorded: BP 90/50 mmHg, HR 57/min, SpO2 99%, and an ECG is performed as shown in the figure. The patient most likely has a lesion involving the</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>A construction worker uses a drill and a pneumatic hammer daily for several hours. The man also presents a radiological lesion characteristic of vibration-induced disease and known as "Kienböck's disease", namely:</t>
+          <t>A construction worker uses a drill and a pneumatic hammer daily for several hours. The man also presents a radiological lesion characteristic of vibration-induced disease and known as "Kienböck's disease", namely</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -5637,7 +5637,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>A 67-year-old woman is found dead by her son in her apartment in Rome. When the Carabinieri arrive, they find her lying supine on the bed with her arms flexed beneath her head. The windows of the house are closed and the ambient temperature is 20 °C. During the on-site investigation, the forensic pathologist measures the body's rectal temperature, which is 36 °C at the start of the investigation and 35.5 °C at the final measurement (about one hour later). Rigor mortis is absent, but faint hypostatic patches are present on the buttocks and shoulders. Externally, there are "suspicious" lesions on the patient's neck and chest that make an autopsy necessary. The findings identified by the forensic pathologist made it possible to determine the time of the woman's death, estimating that death most likely occurred:</t>
+          <t>A 67-year-old woman is found dead by her son in her apartment in Rome. When the Carabinieri arrive, they find her lying supine on the bed with her arms flexed beneath her head. The windows of the house are closed and the ambient temperature is 20 °C. During the on-site investigation, the forensic pathologist measures the body's rectal temperature, which is 36 °C at the start of the investigation and 35.5 °C at the final measurement (about one hour later). Rigor mortis is absent, but faint hypostatic patches are present on the buttocks and shoulders. Externally, there are "suspicious" lesions on the patient's neck and chest that make an autopsy necessary. The findings identified by the forensic pathologist made it possible to determine the time of the woman's death, estimating that death most likely occurred</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>A right-handed patient presents with expressive aphasia characterized by non-fluent spontaneous speech, articulatory difficulties, and buccofacial apraxia. The lesion causing these symptoms is most likely located in the:</t>
+          <t>A right-handed patient presents with expressive aphasia characterized by non-fluent spontaneous speech, articulatory difficulties, and buccofacial apraxia. The lesion causing these symptoms is most likely located in the</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>A 67-year-old patient is referred to the neurologist for rapidly progressive cognitive decline associated with insomnia and irritability. A diagnosis of Creutzfeldt-Jakob disease (CJD) is suspected. The diagnosis is confirmed when cerebrospinal fluid examination shows:</t>
+          <t>A 67-year-old patient is referred to the neurologist for rapidly progressive cognitive decline associated with insomnia and irritability. A diagnosis of Creutzfeldt-Jakob disease (CJD) is suspected. The diagnosis is confirmed when cerebrospinal fluid examination shows</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -6285,7 +6285,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>"A 15-year-old boy is brought to the Emergency Department accompanied by a classmate. The latter is deeply worried because his friend has expressed a wish to die by throwing himself into the Tiber River. Over the past few months he has become gloomy and withdrawn, has stopped seeing his friends, and seems to dwell constantly on the same thoughts: past guilt, death, and feelings of worthlessness. In recent weeks he first developed thoughts of death and then a specific suicide plan. After a thorough evaluation, the neuropsychiatrist considers hospitalization necessary for a probable major depressive disorder with high suicidal risk. The patient, however, refuses hospitalization, stating that he does not need treatment and that he will go to the banks of the Tiber to reflect a little." Based on the available clinical data, the child neuropsychiatrist should:</t>
+          <t>"A 15-year-old boy is brought to the Emergency Department accompanied by a classmate. The latter is deeply worried because his friend has expressed a wish to die by throwing himself into the Tiber River. Over the past few months he has become gloomy and withdrawn, has stopped seeing his friends, and seems to dwell constantly on the same thoughts: past guilt, death, and feelings of worthlessness. In recent weeks he first developed thoughts of death and then a specific suicide plan. After a thorough evaluation, the neuropsychiatrist considers hospitalization necessary for a probable major depressive disorder with high suicidal risk. The patient, however, refuses hospitalization, stating that he does not need treatment and that he will go to the banks of the Tiber to reflect a little." Based on the available clinical data, the child neuropsychiatrist should</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -7745,7 +7745,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>A five-month-old boy, an only child born at term after an uneventful pregnancy. Normal growth. Breastfed. No perinatal problems. For a few days he has had fever (39 °C), loss of appetite, and a few episodes of vomiting. The pediatrician orders a urine culture. In case of a positive urine culture, antibiotic therapy must be administered parenterally:</t>
+          <t>A five-month-old boy, an only child born at term after an uneventful pregnancy. Normal growth. Breastfed. No perinatal problems. For a few days he has had fever (39 °C), loss of appetite, and a few episodes of vomiting. The pediatrician orders a urine culture. In case of a positive urine culture, antibiotic therapy must be administered parenterally</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">

</xml_diff>

<commit_message>
Apply final expert-validated categories to all dataset files
All 1,260 questions now have definitive categories:
- 880 from LLM concordance (Claude = GPT)
- 254 from reviewer concordance (R1 = R2)
- 126 from consensus resolution (in-person discussion)

Applied to IT + EN, JSON + XLSX, per-year + complete.
488 category fields updated across 4 file sets.

Verification: all JSON/XLSX consistent, all categories valid,
IT→EN translation correct for all 1,260 questions.

Updated:
- apply_expert_review.py (rewritten for full pipeline)
- compute_reviewer_agreement.py (updated file paths)
- expert_agreement_report.md (added Section 7: Resolution)
- README.md (resolution documented, folder structure updated)
</commit_message>
<xml_diff>
--- a/Dataset/EN/xlsx/ITAMed_2017_EN.xlsx
+++ b/Dataset/EN/xlsx/ITAMed_2017_EN.xlsx
@@ -710,7 +710,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Gynecology and Obstetrics; Oncology</t>
+          <t>Gynecology and Obstetrics; Infectious Diseases</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Anesthesia and Intensive Care; Cardiology and Cardiac Surgery</t>
+          <t>Cardiology and Cardiac Surgery; General Surgery</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Oncology; Diagnostic Imaging and Nuclear Medicine</t>
+          <t>Pulmonology and Thoracic Surgery; Oncology</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Pulmonology and Thoracic Surgery; Diagnostic Imaging and Nuclear Medicine</t>
+          <t>Pulmonology and Thoracic Surgery; Oncology</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Pulmonology and Thoracic Surgery; Pharmacology and Toxicology</t>
+          <t>Pulmonology and Thoracic Surgery</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Pulmonology and Thoracic Surgery; Oncology</t>
+          <t>Oncology; Pulmonology and Thoracic Surgery</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Pediatrics; General Surgery</t>
+          <t>Pediatrics; Diagnostic Imaging and Nuclear Medicine</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Hygiene, Epidemiology and Statistics; Occupational Medicine</t>
+          <t>Infectious Diseases; Hygiene, Epidemiology and Statistics</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -4018,7 +4018,7 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Pulmonology and Thoracic Surgery; Diagnostic Imaging and Nuclear Medicine</t>
+          <t>Pulmonology and Thoracic Surgery</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -4260,7 +4260,7 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>Cardiology and Cardiac Surgery; Pharmacology and Toxicology</t>
+          <t>Cardiology and Cardiac Surgery</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -4686,7 +4686,7 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>Pulmonology and Thoracic Surgery; Cardiology and Cardiac Surgery</t>
+          <t>Pulmonology and Thoracic Surgery</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
@@ -5092,7 +5092,7 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>Pulmonology and Thoracic Surgery; Gastroenterology</t>
+          <t>Gastroenterology; Pulmonology and Thoracic Surgery</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -5440,7 +5440,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>Endocrinology; Pharmacology and Toxicology</t>
+          <t>Internal Medicine</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>Endocrinology; Nephrology</t>
+          <t>Endocrinology</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
@@ -6020,7 +6020,7 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>Neurology and Neurosurgery; Anesthesia and Intensive Care</t>
+          <t>Neurology and Neurosurgery</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -6552,7 +6552,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Oncology; Gastroenterology</t>
+          <t>Gastroenterology; Oncology</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -6610,7 +6610,7 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Oncology; Pharmacology and Toxicology</t>
+          <t>Oncology</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -6668,7 +6668,7 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>Oncology; Diagnostic Imaging and Nuclear Medicine</t>
+          <t>Oncology; Pulmonology and Thoracic Surgery</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
@@ -7374,7 +7374,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>Endocrinology; Pediatrics</t>
+          <t>Pediatrics; Endocrinology</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -7548,7 +7548,7 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>Endocrinology; Pediatrics</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -7722,7 +7722,7 @@
       </c>
       <c r="K124" t="inlineStr">
         <is>
-          <t>Pediatrics; Urology</t>
+          <t>Pediatrics; Nephrology</t>
         </is>
       </c>
       <c r="L124" t="inlineStr">
@@ -7780,7 +7780,7 @@
       </c>
       <c r="K125" t="inlineStr">
         <is>
-          <t>Pediatrics; Urology</t>
+          <t>Pediatrics; Infectious Diseases</t>
         </is>
       </c>
       <c r="L125" t="inlineStr">
@@ -7896,7 +7896,7 @@
       </c>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Psychiatry; Pharmacology and Toxicology</t>
+          <t>Psychiatry</t>
         </is>
       </c>
       <c r="L127" t="inlineStr">
@@ -8680,7 +8680,7 @@
       </c>
       <c r="K140" t="inlineStr">
         <is>
-          <t>Urology; Diagnostic Imaging and Nuclear Medicine</t>
+          <t>Urology</t>
         </is>
       </c>
       <c r="L140" t="inlineStr">
@@ -8738,7 +8738,7 @@
       </c>
       <c r="K141" t="inlineStr">
         <is>
-          <t>Urology; Pharmacology and Toxicology</t>
+          <t>Urology</t>
         </is>
       </c>
       <c r="L141" t="inlineStr">

</xml_diff>